<commit_message>
added credit card account.
</commit_message>
<xml_diff>
--- a/Personal Budget en-us.xlsx
+++ b/Personal Budget en-us.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rcssi\Code\Personal_Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1F84E09-515A-4E60-B7E3-C3B9F395CFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E2A727-BDB8-4704-A201-A36D894A50F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-114" yWindow="-114" windowWidth="19704" windowHeight="11178" tabRatio="792" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,22 +23,23 @@
   </sheets>
   <definedNames>
     <definedName name="Accounts" localSheetId="5">Goals!#REF!</definedName>
-    <definedName name="Accounts">'Data Validation'!$B$5:$B$8</definedName>
+    <definedName name="Accounts">'Data Validation'!$B$5:$B$9</definedName>
     <definedName name="Dash">'Graphic Annual'!$A$1:$P$26</definedName>
     <definedName name="Discount" localSheetId="5">Goals!#REF!</definedName>
-    <definedName name="Discount">'Data Validation'!$H$5:$H$9</definedName>
+    <definedName name="Discount">'Data Validation'!$F$9:$F$13</definedName>
     <definedName name="Expenses" localSheetId="5">Goals!$D$5:$D$16</definedName>
     <definedName name="Expenses">'Data Validation'!$D$5:$D$16</definedName>
     <definedName name="Income" localSheetId="5">Goals!#REF!</definedName>
-    <definedName name="Income">'Data Validation'!$J$5:$J$9</definedName>
+    <definedName name="Income">'Data Validation'!$H$5:$H$9</definedName>
     <definedName name="Investments" localSheetId="5">Goals!$E$5:$E$6</definedName>
     <definedName name="Investments">'Data Validation'!$F$5:$F$6</definedName>
     <definedName name="Months" localSheetId="5">Goals!#REF!</definedName>
     <definedName name="Months">'Data Validation'!$P$5:$P$16</definedName>
     <definedName name="Net_Salary" localSheetId="5">Goals!#REF!</definedName>
     <definedName name="Net_Salary">'Data Validation'!$N$5:$N$16</definedName>
+    <definedName name="Payment">'Data Validation'!$J$5</definedName>
     <definedName name="Transfer" localSheetId="5">Goals!#REF!</definedName>
-    <definedName name="Transfer">'Data Validation'!$L$5:$L$8</definedName>
+    <definedName name="Transfer">'Data Validation'!$B$5:$B$8</definedName>
     <definedName name="Z_12641207_4FA9_4498_AEA1_9BC1962A4F9A_.wvu.Rows" localSheetId="3" hidden="1">Expenses!$6:$6,Expenses!#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -62,7 +63,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -84,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="89">
   <si>
     <t>Total</t>
   </si>
@@ -345,6 +346,12 @@
   </si>
   <si>
     <t>*Feel free to change the golas and their values as you wish.</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>Payment</t>
   </si>
 </sst>
 </file>
@@ -811,17 +818,17 @@
     <xf numFmtId="44" fontId="3" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -830,7 +837,58 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="19">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1072,8 +1130,8 @@
   <tableStyles count="2" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Tracking table" pivot="0" count="0" xr9:uid="{88815A96-0DF6-4017-8492-6A879ED5C492}"/>
     <tableStyle name="Tracking Table 1" pivot="0" count="2" xr9:uid="{E8395723-409A-4BE8-B2D2-23E4458724D1}">
-      <tableStyleElement type="wholeTable" dxfId="12"/>
-      <tableStyleElement type="headerRow" dxfId="11"/>
+      <tableStyleElement type="wholeTable" dxfId="18"/>
+      <tableStyleElement type="headerRow" dxfId="17"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -9089,7 +9147,7 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>27150</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>90535</xdr:rowOff>
+      <xdr:rowOff>38994</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -9127,7 +9185,7 @@
       <xdr:col>16</xdr:col>
       <xdr:colOff>6</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>42646</xdr:rowOff>
+      <xdr:rowOff>33593</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -9159,13 +9217,13 @@
       <xdr:col>10</xdr:col>
       <xdr:colOff>25610</xdr:colOff>
       <xdr:row>13</xdr:row>
-      <xdr:rowOff>16384</xdr:rowOff>
+      <xdr:rowOff>7331</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>1391</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>87585</xdr:rowOff>
+      <xdr:rowOff>25081</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -9196,21 +9254,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{739BA625-5E32-4F47-8323-C47308DEF24A}" name="Tabela1" displayName="Tabela1" ref="B16:H20" insertRowShift="1" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{739BA625-5E32-4F47-8323-C47308DEF24A}" name="Tabela1" displayName="Tabela1" ref="B16:H20" insertRowShift="1" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="B16:H20" xr:uid="{739BA625-5E32-4F47-8323-C47308DEF24A}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B17:H29">
     <sortCondition ref="B16:B29"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F0A7AC4E-C2B6-48F0-8ABD-146393E8FC69}" name="Date" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{684795FD-753E-4C1F-B63E-5EE124E9D624}" name="Month" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{F0A7AC4E-C2B6-48F0-8ABD-146393E8FC69}" name="Date" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{684795FD-753E-4C1F-B63E-5EE124E9D624}" name="Month" dataDxfId="13">
       <calculatedColumnFormula>IF(ISBLANK(B17),"",PROPER(TEXT(B17,"MMMM")))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{23818CCC-08C7-4066-9B86-98D831460C75}" name="Operation" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{78815540-1C3C-4370-A3E4-1C8E033CFC39}" name="Category" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{F153B94E-6C60-4C63-A86C-8519A94E1F13}" name="Account" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{EE54C9A2-2D53-4D6A-93DF-88B691A8C3D9}" name="Amount" dataDxfId="3" dataCellStyle="Moeda"/>
-    <tableColumn id="5" xr3:uid="{28149A80-D409-4A63-B4C2-6EDA92C21F54}" name="Description" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{23818CCC-08C7-4066-9B86-98D831460C75}" name="Operation" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{78815540-1C3C-4370-A3E4-1C8E033CFC39}" name="Category" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{F153B94E-6C60-4C63-A86C-8519A94E1F13}" name="Account" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{EE54C9A2-2D53-4D6A-93DF-88B691A8C3D9}" name="Amount" dataDxfId="9" dataCellStyle="Moeda"/>
+    <tableColumn id="5" xr3:uid="{28149A80-D409-4A63-B4C2-6EDA92C21F54}" name="Description" dataDxfId="8"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleDark9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9544,10 +9602,10 @@
         <v>35</v>
       </c>
       <c r="H4" s="28" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="J4" s="28" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="L4" s="28" t="s">
         <v>69</v>
@@ -9570,13 +9628,13 @@
         <v>72</v>
       </c>
       <c r="H5" s="73" t="s">
-        <v>51</v>
-      </c>
-      <c r="J5" s="73" t="s">
         <v>47</v>
       </c>
+      <c r="J5" s="74" t="s">
+        <v>87</v>
+      </c>
       <c r="L5" s="74" t="str" cm="1">
-        <f t="array" ref="L5:L8">Accounts</f>
+        <f t="array" ref="L5:L8">Transfer</f>
         <v>Bank 1</v>
       </c>
       <c r="N5" s="74" t="str" cm="1">
@@ -9598,9 +9656,6 @@
         <v>71</v>
       </c>
       <c r="H6" s="73" t="s">
-        <v>50</v>
-      </c>
-      <c r="J6" s="73" t="s">
         <v>48</v>
       </c>
       <c r="L6" s="74" t="str">
@@ -9621,9 +9676,6 @@
         <v>55</v>
       </c>
       <c r="H7" s="73" t="s">
-        <v>66</v>
-      </c>
-      <c r="J7" s="73" t="s">
         <v>68</v>
       </c>
       <c r="L7" s="74" t="str">
@@ -9636,17 +9688,17 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:16" ht="15" x14ac:dyDescent="0.3">
       <c r="B8" s="73" t="s">
         <v>75</v>
       </c>
       <c r="D8" s="73" t="s">
         <v>56</v>
       </c>
+      <c r="F8" s="28" t="s">
+        <v>41</v>
+      </c>
       <c r="H8" s="73" t="s">
-        <v>62</v>
-      </c>
-      <c r="J8" s="73" t="s">
         <v>61</v>
       </c>
       <c r="L8" s="74" t="str">
@@ -9660,13 +9712,16 @@
       </c>
     </row>
     <row r="9" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B9" s="74" t="s">
+        <v>87</v>
+      </c>
       <c r="D9" s="73" t="s">
         <v>53</v>
       </c>
+      <c r="F9" s="73" t="s">
+        <v>51</v>
+      </c>
       <c r="H9" s="73" t="s">
-        <v>52</v>
-      </c>
-      <c r="J9" s="73" t="s">
         <v>49</v>
       </c>
       <c r="N9" s="74" t="str">
@@ -9680,6 +9735,9 @@
       <c r="D10" s="73" t="s">
         <v>5</v>
       </c>
+      <c r="F10" s="73" t="s">
+        <v>50</v>
+      </c>
       <c r="N10" s="74" t="str" cm="1">
         <f t="array" ref="N10:N14">Discount</f>
         <v>Tax I</v>
@@ -9692,6 +9750,9 @@
       <c r="D11" s="73" t="s">
         <v>57</v>
       </c>
+      <c r="F11" s="73" t="s">
+        <v>66</v>
+      </c>
       <c r="N11" s="74" t="str">
         <v>Tax II</v>
       </c>
@@ -9703,6 +9764,9 @@
       <c r="D12" s="73" t="s">
         <v>58</v>
       </c>
+      <c r="F12" s="73" t="s">
+        <v>62</v>
+      </c>
       <c r="N12" s="74" t="str">
         <v>Bank Fee I</v>
       </c>
@@ -9713,6 +9777,9 @@
     <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D13" s="73" t="s">
         <v>65</v>
+      </c>
+      <c r="F13" s="73" t="s">
+        <v>52</v>
       </c>
       <c r="N13" s="74" t="str">
         <v>Bank Fee II</v>
@@ -9887,7 +9954,7 @@
     </row>
     <row r="9" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="15" t="str" cm="1">
-        <f t="array" ref="B9:B12">Accounts</f>
+        <f t="array" ref="B9:B13">Accounts</f>
         <v>Bank 1</v>
       </c>
       <c r="C9" s="36" cm="1">
@@ -9955,25 +10022,30 @@
     </row>
     <row r="13" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="53"/>
-      <c r="B13" s="15" t="s">
+      <c r="B13" s="15" t="str">
+        <v>Credit Card</v>
+      </c>
+      <c r="C13" s="35">
+        <f>SUMIF(Tabela1[Account],B13,Tabela1[Amount])-SUMIF(Tabela1[Category],B13,Tabela1[Amount])</f>
+        <v>0</v>
+      </c>
+      <c r="E13" s="56" t="str">
+        <v>Travel</v>
+      </c>
+      <c r="F13" s="64">
+        <v>0</v>
+      </c>
+      <c r="H13" s="54"/>
+    </row>
+    <row r="14" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="53"/>
+      <c r="B14" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="35">
+      <c r="C14" s="35">
         <f ca="1">ROUND(C5-SUM(C9:C12),2)</f>
         <v>-150</v>
       </c>
-      <c r="E13" s="56" t="str">
-        <v>Travel</v>
-      </c>
-      <c r="F13" s="64">
-        <v>0</v>
-      </c>
-      <c r="H13" s="54"/>
-    </row>
-    <row r="14" spans="1:8" ht="14.3" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="53"/>
-      <c r="B14" s="54"/>
-      <c r="C14" s="54"/>
       <c r="E14" s="56" t="str">
         <v>General expen.</v>
       </c>
@@ -13286,11 +13358,11 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C13">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+  <conditionalFormatting sqref="C13:C14">
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="notEqual">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="notEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13308,7 +13380,7 @@
       <formula1>Accounts</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D17:D20" xr:uid="{0261ACD4-BAB2-4EA0-87AC-74F751F397E2}">
-      <formula1>"Income, Discount, Investments, Expenses, Transfer"</formula1>
+      <formula1>"Income, Discount, Investments, Expenses, Transfer, Payment"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2" xr:uid="{D9270E47-B020-4CBF-A3A9-E523B28C14E7}">
       <formula1>Months</formula1>
@@ -15391,17 +15463,17 @@
       <c r="D5" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="E5" s="83">
+      <c r="E5" s="81">
         <v>450</v>
       </c>
-      <c r="F5" s="84">
-        <f ca="1">$I$5/E5</f>
-        <v>0</v>
-      </c>
-      <c r="H5" s="82" t="s">
-        <v>0</v>
-      </c>
-      <c r="I5" s="83">
+      <c r="F5" s="82">
+        <f t="shared" ref="F5:F16" ca="1" si="0">$I$5/E5</f>
+        <v>0</v>
+      </c>
+      <c r="H5" s="80" t="s">
+        <v>0</v>
+      </c>
+      <c r="I5" s="81">
         <f ca="1">'Balance &amp; Tracking'!C12</f>
         <v>0</v>
       </c>
@@ -15410,11 +15482,11 @@
       <c r="D6" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="83">
+      <c r="E6" s="81">
         <v>350</v>
       </c>
-      <c r="F6" s="84">
-        <f ca="1">$I$5/E6</f>
+      <c r="F6" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15422,11 +15494,11 @@
       <c r="D7" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="E7" s="83">
+      <c r="E7" s="81">
         <v>12000</v>
       </c>
-      <c r="F7" s="84">
-        <f ca="1">$I$5/E7</f>
+      <c r="F7" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15434,11 +15506,11 @@
       <c r="D8" s="73" t="s">
         <v>83</v>
       </c>
-      <c r="E8" s="83">
+      <c r="E8" s="81">
         <v>2500</v>
       </c>
-      <c r="F8" s="84">
-        <f ca="1">$I$5/E8</f>
+      <c r="F8" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15446,11 +15518,11 @@
       <c r="D9" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E9" s="83">
+      <c r="E9" s="81">
         <v>1</v>
       </c>
-      <c r="F9" s="84">
-        <f ca="1">$I$5/E9</f>
+      <c r="F9" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15458,11 +15530,11 @@
       <c r="D10" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E10" s="83">
+      <c r="E10" s="81">
         <v>1</v>
       </c>
-      <c r="F10" s="84">
-        <f ca="1">$I$5/E10</f>
+      <c r="F10" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15470,11 +15542,11 @@
       <c r="D11" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E11" s="83">
+      <c r="E11" s="81">
         <v>1</v>
       </c>
-      <c r="F11" s="84">
-        <f ca="1">$I$5/E11</f>
+      <c r="F11" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15482,11 +15554,11 @@
       <c r="D12" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E12" s="83">
+      <c r="E12" s="81">
         <v>1</v>
       </c>
-      <c r="F12" s="84">
-        <f ca="1">$I$5/E12</f>
+      <c r="F12" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15494,11 +15566,11 @@
       <c r="D13" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E13" s="83">
+      <c r="E13" s="81">
         <v>1</v>
       </c>
-      <c r="F13" s="84">
-        <f ca="1">$I$5/E13</f>
+      <c r="F13" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15506,11 +15578,11 @@
       <c r="D14" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="83">
+      <c r="E14" s="81">
         <v>1</v>
       </c>
-      <c r="F14" s="84">
-        <f ca="1">$I$5/E14</f>
+      <c r="F14" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15518,11 +15590,11 @@
       <c r="D15" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E15" s="83">
+      <c r="E15" s="81">
         <v>1</v>
       </c>
-      <c r="F15" s="84">
-        <f ca="1">$I$5/E15</f>
+      <c r="F15" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15530,11 +15602,11 @@
       <c r="D16" s="73" t="s">
         <v>84</v>
       </c>
-      <c r="E16" s="83">
+      <c r="E16" s="81">
         <v>1</v>
       </c>
-      <c r="F16" s="84">
-        <f ca="1">$I$5/E16</f>
+      <c r="F16" s="82">
+        <f t="shared" ca="1" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -15630,15 +15702,15 @@
       <c r="I2" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="K2" s="80" t="s">
+      <c r="K2" s="83" t="s">
         <v>39</v>
       </c>
-      <c r="L2" s="81"/>
+      <c r="L2" s="84"/>
       <c r="M2" s="24"/>
-      <c r="N2" s="80" t="s">
+      <c r="N2" s="83" t="s">
         <v>45</v>
       </c>
-      <c r="O2" s="81"/>
+      <c r="O2" s="84"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="str" cm="1">

</xml_diff>